<commit_message>
F00: pipeline QC panel and output updates
</commit_message>
<xml_diff>
--- a/04_Figures/F00/c_data/F00_supplementary.xlsx
+++ b/04_Figures/F00/c_data/F00_supplementary.xlsx
@@ -9366,10 +9366,10 @@
         <v>179</v>
       </c>
       <c r="B3" t="n">
-        <v>705</v>
+        <v>608</v>
       </c>
       <c r="C3" t="n">
-        <v>33.3648840511122</v>
+        <v>28.7742546142925</v>
       </c>
     </row>
     <row r="4">
@@ -9377,10 +9377,10 @@
         <v>180</v>
       </c>
       <c r="B4" t="n">
-        <v>446</v>
+        <v>543</v>
       </c>
       <c r="C4" t="n">
-        <v>21.1074301940369</v>
+        <v>25.6980596308566</v>
       </c>
     </row>
   </sheetData>

</xml_diff>